<commit_message>
Corrida | SFE-XCER | 2026-08-21 11:28:53.649736
</commit_message>
<xml_diff>
--- a/indicadores/SFE-XCER_out.xlsx
+++ b/indicadores/SFE-XCER_out.xlsx
@@ -113,13 +113,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">19/08/2026</t>
+    <t xml:space="preserve">21/08/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">pcohan</t>
+    <t xml:space="preserve">arodriguez</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -2226,7 +2226,7 @@
       <c r="B11"/>
       <c r="C11"/>
       <c r="D11" t="n">
-        <v>0.12125268316897</v>
+        <v>0.121252683168969</v>
       </c>
       <c r="E11"/>
       <c r="F11"/>
@@ -2284,7 +2284,7 @@
       <c r="B15"/>
       <c r="C15"/>
       <c r="D15" t="n">
-        <v>0.00932701471157129</v>
+        <v>0.00932701471157139</v>
       </c>
       <c r="E15"/>
       <c r="F15"/>
@@ -2354,7 +2354,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.648616907742487</v>
+        <v>0.64860377321142</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -2384,7 +2384,7 @@
       <c r="B22"/>
       <c r="C22"/>
       <c r="D22" t="n">
-        <v>0.271555295880239</v>
+        <v>0.271714547493877</v>
       </c>
       <c r="E22"/>
       <c r="F22"/>
@@ -27837,7 +27837,7 @@
         <v>531</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>0.0871611620441957</v>
+        <v>0.0871611620441974</v>
       </c>
     </row>
     <row r="6">
@@ -27845,7 +27845,7 @@
         <v>532</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.0785893765575142</v>
+        <v>0.0785893765575149</v>
       </c>
     </row>
     <row r="7">
@@ -27853,7 +27853,7 @@
         <v>533</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.0459600111444907</v>
+        <v>0.0459600111444914</v>
       </c>
     </row>
     <row r="8">
@@ -27861,7 +27861,7 @@
         <v>534</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>-0.00839511299741596</v>
+        <v>-0.00839511299741496</v>
       </c>
     </row>
     <row r="9">
@@ -27869,7 +27869,7 @@
         <v>535</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>-0.0199665149644856</v>
+        <v>-0.0199665149644863</v>
       </c>
     </row>
     <row r="10">
@@ -27877,7 +27877,7 @@
         <v>536</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>-0.00289001625200092</v>
+        <v>-0.00289001625200345</v>
       </c>
     </row>
     <row r="11">
@@ -27885,7 +27885,7 @@
         <v>537</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>-0.00290604547848592</v>
+        <v>-0.0029060454784885</v>
       </c>
     </row>
     <row r="12">
@@ -27893,7 +27893,7 @@
         <v>538</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.0423500471752307</v>
+        <v>0.04235004717523</v>
       </c>
     </row>
     <row r="13">
@@ -27909,7 +27909,7 @@
         <v>540</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.0965764707968317</v>
+        <v>0.0965764707968323</v>
       </c>
     </row>
     <row r="15">
@@ -27917,7 +27917,7 @@
         <v>541</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.0610284440870361</v>
+        <v>0.0610284440870364</v>
       </c>
     </row>
     <row r="16">
@@ -27925,7 +27925,7 @@
         <v>542</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.0189481378739266</v>
+        <v>0.0189481378739257</v>
       </c>
     </row>
     <row r="17">
@@ -27933,7 +27933,7 @@
         <v>543</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>-0.0177813106102326</v>
+        <v>-0.0177813106102345</v>
       </c>
     </row>
     <row r="18">
@@ -27941,7 +27941,7 @@
         <v>544</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>-0.0324035736519851</v>
+        <v>-0.0324035736519868</v>
       </c>
     </row>
     <row r="19">
@@ -27949,7 +27949,7 @@
         <v>545</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.0117149049687428</v>
+        <v>0.0117149049687416</v>
       </c>
     </row>
     <row r="20">
@@ -27957,7 +27957,7 @@
         <v>546</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.0739742137114314</v>
+        <v>0.0739742137114309</v>
       </c>
     </row>
     <row r="21">
@@ -27965,7 +27965,7 @@
         <v>547</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>0.110581172294761</v>
+        <v>0.11058117229476</v>
       </c>
     </row>
     <row r="22">
@@ -27973,7 +27973,7 @@
         <v>548</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>0.12125268316897</v>
+        <v>0.121252683168969</v>
       </c>
     </row>
     <row r="23">
@@ -27981,7 +27981,7 @@
         <v>549</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>0.086565664241755</v>
+        <v>0.0865656642417551</v>
       </c>
     </row>
     <row r="24">

</xml_diff>